<commit_message>
magpul type1/2 rail panels + mlok hand stop set
</commit_message>
<xml_diff>
--- a/changes/foregrips.xlsx
+++ b/changes/foregrips.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yifan\Documents\deadline-balancing\changes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\whyth\Documents\GitHub\deadline-balancing\changes\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AEF22A4-9E5D-4AFD-BE0D-DF3462A8EC65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6813540-92AB-4717-903A-B86E9B209CE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="foregrips" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="148">
   <si>
     <t>new</t>
   </si>
@@ -459,13 +459,31 @@
   </si>
   <si>
     <t>Magtap MCP MAG597</t>
+  </si>
+  <si>
+    <t>magtap_mlok_hand_stop</t>
+  </si>
+  <si>
+    <t>Magtap MLOK Hand Stop</t>
+  </si>
+  <si>
+    <t>magtap_mlok_index_panel</t>
+  </si>
+  <si>
+    <t>Magtap MLOK Index Panel</t>
+  </si>
+  <si>
+    <t>magtap_mlok_index_panel_flipped</t>
+  </si>
+  <si>
+    <t>Magtap MLOK Index Panel Flipped</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -475,94 +493,117 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="18"/>
       <color theme="3"/>
       <name val="Calibri Light"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="15"/>
       <color theme="3"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="13"/>
       <color theme="3"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="3"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF9C5700"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="11"/>
       <color rgb="FF7F7F7F"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="0"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Consolas"/>
+      <family val="3"/>
     </font>
   </fonts>
   <fills count="33">
@@ -906,8 +947,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
@@ -1161,7 +1203,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:S71"/>
+  <dimension ref="A1:S74"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="29.140625" customWidth="1"/>
@@ -1253,7 +1295,7 @@
         <v>400</v>
       </c>
       <c r="N3">
-        <f t="shared" ref="N3:N71" si="0">C3-D3*20-E3*0.8-F3*0.6</f>
+        <f>C3-D3*20-E3*0.8-F3*0.6</f>
         <v>7.1999999999999993</v>
       </c>
     </row>
@@ -1280,7 +1322,7 @@
         <v>300</v>
       </c>
       <c r="N4">
-        <f t="shared" si="0"/>
+        <f>C4-D4*20-E4*0.8-F4*0.6</f>
         <v>7</v>
       </c>
     </row>
@@ -1334,7 +1376,7 @@
         <v>800</v>
       </c>
       <c r="N6">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="N3:N74" si="0">C6-D6*20-E6*0.8-F6*0.6</f>
         <v>5.1999999999999993</v>
       </c>
     </row>
@@ -1577,7 +1619,7 @@
         <v>300</v>
       </c>
       <c r="N15">
-        <f t="shared" si="0"/>
+        <f>C15-D15*20-E15*0.8-F15*0.6</f>
         <v>7</v>
       </c>
     </row>
@@ -1604,7 +1646,7 @@
         <v>600</v>
       </c>
       <c r="N16">
-        <f t="shared" si="0"/>
+        <f>C16-D16*20-E16*0.8-F16*0.6</f>
         <v>6.8</v>
       </c>
     </row>
@@ -1635,99 +1677,99 @@
         <v>6.3999999999999995</v>
       </c>
     </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B18" t="s">
+        <v>143</v>
+      </c>
+      <c r="C18">
+        <v>6</v>
+      </c>
+      <c r="D18">
+        <v>0.03</v>
+      </c>
+      <c r="E18">
+        <v>-2</v>
+      </c>
+      <c r="F18">
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <v>600</v>
+      </c>
+      <c r="N18">
+        <f t="shared" ref="N18:N20" si="1">C18-D18*20-E18*0.8-F18*0.6</f>
+        <v>7</v>
+      </c>
+    </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>42</v>
+      <c r="A19" s="1" t="s">
+        <v>144</v>
       </c>
       <c r="B19" t="s">
-        <v>20</v>
+        <v>145</v>
       </c>
       <c r="C19">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D19">
-        <v>0.15</v>
+        <v>0.02</v>
       </c>
       <c r="E19">
         <v>0</v>
       </c>
       <c r="F19">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="M19">
-        <v>1100</v>
+        <v>500</v>
       </c>
       <c r="N19">
-        <f t="shared" si="0"/>
-        <v>-3</v>
+        <f t="shared" si="1"/>
+        <v>6.1999999999999993</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>43</v>
+        <v>146</v>
       </c>
       <c r="B20" t="s">
-        <v>21</v>
+        <v>147</v>
       </c>
       <c r="C20">
+        <v>6</v>
+      </c>
+      <c r="D20">
+        <v>0.02</v>
+      </c>
+      <c r="E20">
+        <v>0</v>
+      </c>
+      <c r="F20">
         <v>-1</v>
       </c>
-      <c r="D20">
-        <v>0.09</v>
-      </c>
-      <c r="E20">
-        <v>-4</v>
-      </c>
-      <c r="F20">
-        <v>-5</v>
-      </c>
       <c r="M20">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="N20">
-        <f>C20-D20*20-E20*0.8-F20*0.6</f>
-        <v>3.4000000000000004</v>
-      </c>
-    </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>44</v>
-      </c>
-      <c r="B21" t="s">
-        <v>22</v>
-      </c>
-      <c r="C21">
-        <v>-3</v>
-      </c>
-      <c r="D21">
-        <v>0.09</v>
-      </c>
-      <c r="E21">
-        <v>-6</v>
-      </c>
-      <c r="F21">
-        <v>-7</v>
-      </c>
-      <c r="M21">
-        <v>0</v>
-      </c>
-      <c r="N21">
-        <f t="shared" si="0"/>
-        <v>4.2000000000000011</v>
+        <f t="shared" si="1"/>
+        <v>6.1999999999999993</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B22" t="s">
-        <v>105</v>
+        <v>20</v>
       </c>
       <c r="C22">
         <v>0</v>
       </c>
       <c r="D22">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -1736,463 +1778,463 @@
         <v>0</v>
       </c>
       <c r="M22">
-        <v>700</v>
+        <v>1100</v>
       </c>
       <c r="N22">
         <f t="shared" si="0"/>
-        <v>-2</v>
+        <v>-3</v>
       </c>
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B23" t="s">
-        <v>106</v>
+        <v>21</v>
       </c>
       <c r="C23">
         <v>-1</v>
       </c>
       <c r="D23">
-        <v>0.06</v>
+        <v>0.09</v>
       </c>
       <c r="E23">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="F23">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="M23">
         <v>0</v>
       </c>
       <c r="N23">
-        <f t="shared" si="0"/>
-        <v>2.6</v>
+        <f>C23-D23*20-E23*0.8-F23*0.6</f>
+        <v>3.4000000000000004</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B24" t="s">
-        <v>107</v>
+        <v>22</v>
       </c>
       <c r="C24">
         <v>-3</v>
       </c>
       <c r="D24">
-        <v>0.06</v>
+        <v>0.09</v>
       </c>
       <c r="E24">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="F24">
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="M24">
         <v>0</v>
       </c>
       <c r="N24">
         <f t="shared" si="0"/>
-        <v>3.3999999999999995</v>
+        <v>4.2000000000000011</v>
       </c>
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="B25" t="s">
-        <v>23</v>
+        <v>105</v>
       </c>
       <c r="C25">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="D25">
-        <v>0.23</v>
+        <v>0.1</v>
       </c>
       <c r="E25">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="F25">
-        <v>-3</v>
+        <v>0</v>
       </c>
       <c r="M25">
-        <v>1000</v>
+        <v>700</v>
       </c>
       <c r="N25">
         <f t="shared" si="0"/>
-        <v>3.9999999999999991</v>
+        <v>-2</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B26" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C26">
-        <v>6</v>
+        <v>-1</v>
       </c>
       <c r="D26">
-        <v>0.23</v>
+        <v>0.06</v>
       </c>
       <c r="E26">
         <v>-3</v>
       </c>
       <c r="F26">
+        <v>-4</v>
+      </c>
+      <c r="M26">
         <v>0</v>
       </c>
-      <c r="M26">
-        <v>1500</v>
-      </c>
       <c r="N26">
         <f t="shared" si="0"/>
-        <v>3.8</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="B27" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C27">
-        <v>1</v>
+        <v>-3</v>
       </c>
       <c r="D27">
-        <v>0.16</v>
+        <v>0.06</v>
       </c>
       <c r="E27">
-        <v>-1</v>
+        <v>-5</v>
       </c>
       <c r="F27">
-        <v>-7</v>
+        <v>-6</v>
       </c>
       <c r="M27">
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="N27">
         <f t="shared" si="0"/>
-        <v>2.8</v>
+        <v>3.3999999999999995</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B28" t="s">
-        <v>110</v>
+        <v>23</v>
       </c>
       <c r="C28">
         <v>6</v>
       </c>
       <c r="D28">
-        <v>0.09</v>
+        <v>0.23</v>
       </c>
       <c r="E28">
-        <v>-2</v>
+        <v>-1</v>
       </c>
       <c r="F28">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="M28">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="N28">
         <f t="shared" si="0"/>
-        <v>7.0000000000000009</v>
+        <v>3.9999999999999991</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B29" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="C29">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D29">
-        <v>0.11</v>
+        <v>0.23</v>
       </c>
       <c r="E29">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="F29">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="M29">
-        <v>400</v>
+        <v>1500</v>
       </c>
       <c r="N29">
         <f t="shared" si="0"/>
-        <v>6.6</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="B30" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C30">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D30">
-        <v>0.09</v>
+        <v>0.16</v>
       </c>
       <c r="E30">
-        <v>-6</v>
+        <v>-1</v>
       </c>
       <c r="F30">
-        <v>-3</v>
+        <v>-7</v>
       </c>
       <c r="M30">
-        <v>700</v>
+        <v>900</v>
       </c>
       <c r="N30">
         <f t="shared" si="0"/>
-        <v>6.8000000000000007</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B31" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="C31">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D31">
         <v>0.09</v>
       </c>
       <c r="E31">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="F31">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="M31">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="N31">
         <f t="shared" si="0"/>
-        <v>7.2</v>
+        <v>7.0000000000000009</v>
       </c>
     </row>
     <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>138</v>
+        <v>52</v>
       </c>
       <c r="B32" t="s">
-        <v>139</v>
+        <v>111</v>
       </c>
       <c r="C32">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D32">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
       <c r="E32">
-        <v>-2</v>
+        <v>-4</v>
       </c>
       <c r="F32">
-        <v>-5</v>
+        <v>-1</v>
       </c>
       <c r="M32">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="N32">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="B33" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C33">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D33">
-        <v>0.1</v>
+        <v>0.09</v>
       </c>
       <c r="E33">
         <v>-6</v>
       </c>
       <c r="F33">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="M33">
-        <v>400</v>
+        <v>700</v>
       </c>
       <c r="N33">
         <f t="shared" si="0"/>
-        <v>7.0000000000000009</v>
+        <v>6.8000000000000007</v>
       </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B34" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C34">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D34">
-        <v>0.11</v>
+        <v>0.09</v>
       </c>
       <c r="E34">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="F34">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="M34">
-        <v>800</v>
+        <v>600</v>
       </c>
       <c r="N34">
         <f t="shared" si="0"/>
-        <v>5.1999999999999993</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>57</v>
+        <v>138</v>
       </c>
       <c r="B35" t="s">
-        <v>116</v>
+        <v>139</v>
       </c>
       <c r="C35">
         <v>4</v>
       </c>
       <c r="D35">
-        <v>7.0000000000000007E-2</v>
+        <v>0.08</v>
       </c>
       <c r="E35">
         <v>-2</v>
       </c>
       <c r="F35">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="M35">
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="N35">
         <f t="shared" si="0"/>
-        <v>6.6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="B36" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C36">
         <v>3</v>
       </c>
       <c r="D36">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="E36">
-        <v>-5</v>
+        <v>-6</v>
       </c>
       <c r="F36">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="M36">
-        <v>600</v>
+        <v>400</v>
       </c>
       <c r="N36">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>7.0000000000000009</v>
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B37" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="C37">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D37">
-        <v>7.0000000000000007E-2</v>
+        <v>0.11</v>
       </c>
       <c r="E37">
-        <v>-3</v>
+        <v>-5</v>
       </c>
       <c r="F37">
-        <v>-3</v>
+        <v>-4</v>
       </c>
       <c r="M37">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="N37">
         <f t="shared" si="0"/>
-        <v>6.8</v>
+        <v>5.1999999999999993</v>
       </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B38" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C38">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D38">
-        <v>0.1</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E38">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="F38">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="M38">
-        <v>400</v>
+        <v>600</v>
       </c>
       <c r="N38">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B39" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="C39">
         <v>3</v>
       </c>
       <c r="D39">
-        <v>0.08</v>
+        <v>0.09</v>
       </c>
       <c r="E39">
-        <v>-4</v>
+        <v>-5</v>
       </c>
       <c r="F39">
-        <v>-4</v>
+        <v>-3</v>
       </c>
       <c r="M39">
         <v>600</v>
@@ -2204,52 +2246,52 @@
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B40" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C40">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D40">
-        <v>0.1</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E40">
         <v>-3</v>
       </c>
       <c r="F40">
-        <v>-5</v>
+        <v>-3</v>
       </c>
       <c r="M40">
-        <v>700</v>
+        <v>300</v>
       </c>
       <c r="N40">
         <f t="shared" si="0"/>
-        <v>6.4</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B41" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C41">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D41">
-        <v>0.05</v>
+        <v>0.1</v>
       </c>
       <c r="E41">
-        <v>-1</v>
+        <v>-5</v>
       </c>
       <c r="F41">
-        <v>-2</v>
+        <v>-5</v>
       </c>
       <c r="M41">
-        <v>700</v>
+        <v>400</v>
       </c>
       <c r="N41">
         <f t="shared" si="0"/>
@@ -2258,450 +2300,450 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B42" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C42">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D42">
-        <v>0.15</v>
+        <v>0.08</v>
       </c>
       <c r="E42">
-        <v>-6</v>
+        <v>-4</v>
       </c>
       <c r="F42">
-        <v>-1</v>
+        <v>-4</v>
       </c>
       <c r="M42">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="N42">
         <f t="shared" si="0"/>
-        <v>6.4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="43" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B43" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C43">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D43">
         <v>0.1</v>
       </c>
       <c r="E43">
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="F43">
         <v>-5</v>
       </c>
       <c r="M43">
-        <v>300</v>
+        <v>700</v>
       </c>
       <c r="N43">
         <f t="shared" si="0"/>
-        <v>6.8</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="44" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B44" t="s">
-        <v>24</v>
+        <v>121</v>
       </c>
       <c r="C44">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D44">
-        <v>0.09</v>
+        <v>0.05</v>
       </c>
       <c r="E44">
+        <v>-1</v>
+      </c>
+      <c r="F44">
         <v>-2</v>
       </c>
-      <c r="F44">
-        <v>-4</v>
-      </c>
       <c r="M44">
-        <v>800</v>
+        <v>700</v>
       </c>
       <c r="N44">
         <f t="shared" si="0"/>
-        <v>7.2000000000000011</v>
+        <v>7</v>
       </c>
     </row>
     <row r="45" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B45" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C45">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D45">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="E45">
-        <v>-4</v>
+        <v>-6</v>
       </c>
       <c r="F45">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="M45">
         <v>500</v>
       </c>
       <c r="N45">
         <f t="shared" si="0"/>
-        <v>7</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="46" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B46" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C46">
         <v>5</v>
       </c>
       <c r="D46">
-        <v>7.0000000000000007E-2</v>
+        <v>0.1</v>
       </c>
       <c r="E46">
-        <v>-3</v>
+        <v>-1</v>
       </c>
       <c r="F46">
-        <v>-2</v>
+        <v>-5</v>
       </c>
       <c r="M46">
         <v>300</v>
       </c>
       <c r="N46">
         <f t="shared" si="0"/>
-        <v>7.2</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="47" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B47" t="s">
-        <v>126</v>
+        <v>24</v>
       </c>
       <c r="C47">
         <v>5</v>
       </c>
       <c r="D47">
-        <v>7.0000000000000007E-2</v>
+        <v>0.09</v>
       </c>
       <c r="E47">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="F47">
-        <v>-2</v>
+        <v>-4</v>
       </c>
       <c r="M47">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="N47">
         <f t="shared" si="0"/>
-        <v>7.2</v>
+        <v>7.2000000000000011</v>
       </c>
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B48" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C48">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D48">
-        <v>0.05</v>
+        <v>0.06</v>
       </c>
       <c r="E48">
-        <v>-2</v>
+        <v>-4</v>
       </c>
       <c r="F48">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="M48">
-        <v>300</v>
+        <v>500</v>
       </c>
       <c r="N48">
         <f t="shared" si="0"/>
-        <v>7.1999999999999993</v>
+        <v>7</v>
       </c>
     </row>
     <row r="49" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B49" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C49">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D49">
-        <v>0.05</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E49">
+        <v>-3</v>
+      </c>
+      <c r="F49">
         <v>-2</v>
-      </c>
-      <c r="F49">
-        <v>-1</v>
       </c>
       <c r="M49">
         <v>300</v>
       </c>
       <c r="N49">
         <f t="shared" si="0"/>
-        <v>7.1999999999999993</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="50" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B50" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C50">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D50">
-        <v>0.09</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E50">
         <v>-3</v>
       </c>
       <c r="F50">
-        <v>-4</v>
+        <v>-2</v>
       </c>
       <c r="M50">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="N50">
         <f t="shared" si="0"/>
-        <v>7</v>
-      </c>
-      <c r="P50">
-        <v>35</v>
-      </c>
-      <c r="Q50">
-        <f>P50*8+100</f>
-        <v>380</v>
-      </c>
-      <c r="R50">
-        <v>2.4</v>
-      </c>
-      <c r="S50">
-        <f>R50*3*0.01+0.01</f>
-        <v>8.199999999999999E-2</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="51" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>70</v>
+      </c>
+      <c r="B51" t="s">
+        <v>127</v>
+      </c>
+      <c r="C51">
+        <v>6</v>
+      </c>
+      <c r="D51">
+        <v>0.05</v>
+      </c>
+      <c r="E51">
+        <v>-2</v>
+      </c>
+      <c r="F51">
+        <v>-1</v>
+      </c>
+      <c r="M51">
+        <v>300</v>
+      </c>
       <c r="N51">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>7.1999999999999993</v>
       </c>
     </row>
     <row r="52" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B52" t="s">
-        <v>25</v>
+        <v>128</v>
       </c>
       <c r="C52">
+        <v>6</v>
+      </c>
+      <c r="D52">
+        <v>0.05</v>
+      </c>
+      <c r="E52">
+        <v>-2</v>
+      </c>
+      <c r="F52">
         <v>-1</v>
       </c>
-      <c r="D52">
-        <v>0.03</v>
-      </c>
-      <c r="E52">
-        <v>0</v>
-      </c>
-      <c r="F52">
-        <v>0</v>
-      </c>
       <c r="M52">
-        <v>500</v>
+        <v>300</v>
       </c>
       <c r="N52">
         <f t="shared" si="0"/>
-        <v>-1.6</v>
+        <v>7.1999999999999993</v>
       </c>
     </row>
     <row r="53" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B53" t="s">
-        <v>26</v>
+        <v>129</v>
       </c>
       <c r="C53">
-        <v>-0.5</v>
+        <v>4</v>
       </c>
       <c r="D53">
-        <v>0.03</v>
+        <v>0.09</v>
       </c>
       <c r="E53">
+        <v>-3</v>
+      </c>
+      <c r="F53">
+        <v>-4</v>
+      </c>
+      <c r="M53">
+        <v>500</v>
+      </c>
+      <c r="N53">
+        <f t="shared" si="0"/>
+        <v>7</v>
+      </c>
+      <c r="P53">
+        <v>35</v>
+      </c>
+      <c r="Q53">
+        <f>P53*8+100</f>
+        <v>380</v>
+      </c>
+      <c r="R53">
+        <v>2.4</v>
+      </c>
+      <c r="S53">
+        <f>R53*3*0.01+0.01</f>
+        <v>8.199999999999999E-2</v>
+      </c>
+    </row>
+    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="N54">
+        <f t="shared" si="0"/>
         <v>0</v>
-      </c>
-      <c r="F53">
-        <v>0</v>
-      </c>
-      <c r="M53">
-        <v>200</v>
-      </c>
-      <c r="N53">
-        <f t="shared" si="0"/>
-        <v>-1.1000000000000001</v>
-      </c>
-    </row>
-    <row r="54" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>75</v>
-      </c>
-      <c r="B54" t="s">
-        <v>27</v>
-      </c>
-      <c r="C54">
-        <v>-0.5</v>
-      </c>
-      <c r="D54">
-        <v>0.02</v>
-      </c>
-      <c r="E54">
-        <v>0</v>
-      </c>
-      <c r="F54">
-        <v>0</v>
-      </c>
-      <c r="M54">
-        <v>200</v>
-      </c>
-      <c r="N54">
-        <f t="shared" si="0"/>
-        <v>-0.9</v>
       </c>
     </row>
     <row r="55" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B55" t="s">
-        <v>130</v>
+        <v>25</v>
       </c>
       <c r="C55">
-        <v>3</v>
+        <v>-1</v>
       </c>
       <c r="D55">
-        <v>0.05</v>
+        <v>0.03</v>
       </c>
       <c r="E55">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="F55">
-        <v>-7</v>
+        <v>0</v>
       </c>
       <c r="M55">
         <v>500</v>
       </c>
       <c r="N55">
         <f t="shared" si="0"/>
-        <v>7.8000000000000007</v>
+        <v>-1.6</v>
       </c>
     </row>
     <row r="56" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B56" t="s">
-        <v>131</v>
+        <v>26</v>
       </c>
       <c r="C56">
-        <v>1</v>
+        <v>-0.5</v>
       </c>
       <c r="D56">
-        <v>7.0000000000000007E-2</v>
+        <v>0.03</v>
       </c>
       <c r="E56">
-        <v>-4</v>
+        <v>0</v>
       </c>
       <c r="F56">
-        <v>-8</v>
+        <v>0</v>
       </c>
       <c r="M56">
-        <v>600</v>
+        <v>200</v>
       </c>
       <c r="N56">
         <f t="shared" si="0"/>
-        <v>7.6</v>
+        <v>-1.1000000000000001</v>
       </c>
     </row>
     <row r="57" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B57" t="s">
-        <v>132</v>
+        <v>27</v>
       </c>
       <c r="C57">
-        <v>-1</v>
+        <v>-0.5</v>
       </c>
       <c r="D57">
-        <v>0.1</v>
+        <v>0.02</v>
       </c>
       <c r="E57">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="F57">
-        <v>-9</v>
+        <v>0</v>
       </c>
       <c r="M57">
-        <v>700</v>
+        <v>200</v>
       </c>
       <c r="N57">
         <f t="shared" si="0"/>
-        <v>6.3999999999999995</v>
+        <v>-0.9</v>
       </c>
     </row>
     <row r="58" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="B58" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C58">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D58">
         <v>0.05</v>
       </c>
       <c r="E58">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="F58">
-        <v>-4</v>
+        <v>-7</v>
       </c>
       <c r="M58">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="N58">
         <f t="shared" si="0"/>
@@ -2710,25 +2752,25 @@
     </row>
     <row r="59" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B59" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C59">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D59">
-        <v>0.05</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E59">
         <v>-4</v>
       </c>
       <c r="F59">
-        <v>-4</v>
+        <v>-8</v>
       </c>
       <c r="M59">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="N59">
         <f t="shared" si="0"/>
@@ -2737,52 +2779,52 @@
     </row>
     <row r="60" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B60" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C60">
-        <v>5</v>
+        <v>-1</v>
       </c>
       <c r="D60">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E60">
-        <v>-2</v>
+        <v>-5</v>
       </c>
       <c r="F60">
-        <v>-3</v>
+        <v>-9</v>
       </c>
       <c r="M60">
-        <v>500</v>
+        <v>700</v>
       </c>
       <c r="N60">
         <f t="shared" si="0"/>
-        <v>7.6000000000000005</v>
+        <v>6.3999999999999995</v>
       </c>
     </row>
     <row r="61" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B61" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="C61">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D61">
         <v>0.05</v>
       </c>
       <c r="E61">
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="F61">
-        <v>-7</v>
+        <v>-4</v>
       </c>
       <c r="M61">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="N61">
         <f t="shared" si="0"/>
@@ -2791,25 +2833,25 @@
     </row>
     <row r="62" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B62" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C62">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D62">
-        <v>7.0000000000000007E-2</v>
+        <v>0.05</v>
       </c>
       <c r="E62">
         <v>-4</v>
       </c>
       <c r="F62">
-        <v>-8</v>
+        <v>-4</v>
       </c>
       <c r="M62">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="N62">
         <f t="shared" si="0"/>
@@ -2818,52 +2860,52 @@
     </row>
     <row r="63" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B63" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C63">
-        <v>-1</v>
+        <v>5</v>
       </c>
       <c r="D63">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E63">
-        <v>-5</v>
+        <v>-2</v>
       </c>
       <c r="F63">
-        <v>-9</v>
+        <v>-3</v>
       </c>
       <c r="M63">
-        <v>700</v>
+        <v>500</v>
       </c>
       <c r="N63">
         <f t="shared" si="0"/>
-        <v>6.3999999999999995</v>
+        <v>7.6000000000000005</v>
       </c>
     </row>
     <row r="64" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B64" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C64">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D64">
         <v>0.05</v>
       </c>
       <c r="E64">
-        <v>-3</v>
+        <v>-2</v>
       </c>
       <c r="F64">
-        <v>-4</v>
+        <v>-7</v>
       </c>
       <c r="M64">
-        <v>600</v>
+        <v>500</v>
       </c>
       <c r="N64">
         <f t="shared" si="0"/>
@@ -2872,25 +2914,25 @@
     </row>
     <row r="65" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B65" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C65">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D65">
-        <v>0.05</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="E65">
         <v>-4</v>
       </c>
       <c r="F65">
-        <v>-4</v>
+        <v>-8</v>
       </c>
       <c r="M65">
-        <v>500</v>
+        <v>600</v>
       </c>
       <c r="N65">
         <f t="shared" si="0"/>
@@ -2899,92 +2941,110 @@
     </row>
     <row r="66" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B66" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C66">
-        <v>5</v>
+        <v>-1</v>
       </c>
       <c r="D66">
-        <v>0.04</v>
+        <v>0.1</v>
       </c>
       <c r="E66">
-        <v>-2</v>
+        <v>-5</v>
       </c>
       <c r="F66">
+        <v>-9</v>
+      </c>
+      <c r="M66">
+        <v>700</v>
+      </c>
+      <c r="N66">
+        <f t="shared" si="0"/>
+        <v>6.3999999999999995</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>85</v>
+      </c>
+      <c r="B67" t="s">
+        <v>133</v>
+      </c>
+      <c r="C67">
+        <v>4</v>
+      </c>
+      <c r="D67">
+        <v>0.05</v>
+      </c>
+      <c r="E67">
         <v>-3</v>
       </c>
-      <c r="M66">
-        <v>500</v>
-      </c>
-      <c r="N66">
-        <f t="shared" si="0"/>
-        <v>7.6000000000000005</v>
-      </c>
-    </row>
-    <row r="67" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="F67">
+        <v>-4</v>
+      </c>
+      <c r="M67">
+        <v>600</v>
+      </c>
       <c r="N67">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>7.8000000000000007</v>
       </c>
     </row>
     <row r="68" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B68" t="s">
-        <v>28</v>
+        <v>134</v>
       </c>
       <c r="C68">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D68">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="E68">
-        <v>-5</v>
+        <v>-4</v>
       </c>
       <c r="F68">
         <v>-4</v>
       </c>
       <c r="M68">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="N68">
         <f t="shared" si="0"/>
-        <v>6.4</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="69" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B69" t="s">
-        <v>29</v>
+        <v>135</v>
       </c>
       <c r="C69">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D69">
-        <v>0.1</v>
+        <v>0.04</v>
       </c>
       <c r="E69">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="F69">
-        <v>0</v>
-      </c>
-      <c r="H69">
-        <v>0.2</v>
+        <v>-3</v>
       </c>
       <c r="M69">
-        <v>0</v>
+        <v>500</v>
       </c>
       <c r="N69">
-        <f>C69-D69*20-E69*0.8-F69*0.6-H69*2</f>
-        <v>3</v>
+        <f t="shared" si="0"/>
+        <v>7.6000000000000005</v>
       </c>
     </row>
     <row r="70" spans="1:14" x14ac:dyDescent="0.25">
@@ -2995,27 +3055,90 @@
     </row>
     <row r="71" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B71" t="s">
-        <v>136</v>
+        <v>28</v>
       </c>
       <c r="C71">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D71">
         <v>0.1</v>
       </c>
       <c r="E71">
+        <v>-5</v>
+      </c>
+      <c r="F71">
+        <v>-4</v>
+      </c>
+      <c r="M71">
+        <v>0</v>
+      </c>
+      <c r="N71">
+        <f t="shared" si="0"/>
+        <v>6.4</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>89</v>
+      </c>
+      <c r="B72" t="s">
+        <v>29</v>
+      </c>
+      <c r="C72">
+        <v>7</v>
+      </c>
+      <c r="D72">
+        <v>0.1</v>
+      </c>
+      <c r="E72">
+        <v>2</v>
+      </c>
+      <c r="F72">
+        <v>0</v>
+      </c>
+      <c r="H72">
+        <v>0.2</v>
+      </c>
+      <c r="M72">
+        <v>0</v>
+      </c>
+      <c r="N72">
+        <f>C72-D72*20-E72*0.8-F72*0.6-H72*2</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="N73">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>90</v>
+      </c>
+      <c r="B74" t="s">
+        <v>136</v>
+      </c>
+      <c r="C74">
+        <v>3</v>
+      </c>
+      <c r="D74">
+        <v>0.1</v>
+      </c>
+      <c r="E74">
         <v>-2</v>
       </c>
-      <c r="F71">
+      <c r="F74">
         <v>-2</v>
       </c>
-      <c r="M71">
+      <c r="M74">
         <v>800</v>
       </c>
-      <c r="N71">
+      <c r="N74">
         <f t="shared" si="0"/>
         <v>3.8</v>
       </c>

</xml_diff>